<commit_message>
add component-level coupling of cost and ghg data
</commit_message>
<xml_diff>
--- a/data/component_cost_lca_data.xlsx
+++ b/data/component_cost_lca_data.xlsx
@@ -8,22 +8,23 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\github\building_impact_model\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99173236-ECB2-4DB3-9F24-9A63255B2534}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0440BE1C-3294-417F-9EBE-1E3C544A6702}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="RS_Means_BC_Cost_Data" sheetId="10" r:id="rId1"/>
-    <sheet name="All_LCA_Data" sheetId="11" r:id="rId2"/>
-    <sheet name="Cost_LCA_Coupled" sheetId="12" r:id="rId3"/>
-    <sheet name="test_fp" sheetId="16" r:id="rId4"/>
-    <sheet name="test_comp" sheetId="17" r:id="rId5"/>
-    <sheet name="USEEIO_data" sheetId="15" r:id="rId6"/>
-    <sheet name="HVAC_systems" sheetId="13" r:id="rId7"/>
+    <sheet name="component_list" sheetId="18" r:id="rId1"/>
+    <sheet name="RS_Means_BC_Cost_Data" sheetId="10" r:id="rId2"/>
+    <sheet name="All_LCA_Data" sheetId="11" r:id="rId3"/>
+    <sheet name="Cost_LCA_Coupled" sheetId="12" r:id="rId4"/>
+    <sheet name="test_fp" sheetId="16" r:id="rId5"/>
+    <sheet name="test_comp" sheetId="17" r:id="rId6"/>
+    <sheet name="USEEIO_data" sheetId="15" r:id="rId7"/>
+    <sheet name="HVAC_systems" sheetId="13" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">All_LCA_Data!$A$1:$M$195</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">RS_Means_BC_Cost_Data!$A$1:$I$304</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">All_LCA_Data!$A$1:$M$195</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">RS_Means_BC_Cost_Data!$A$1:$I$304</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -46,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8343" uniqueCount="1803">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8381" uniqueCount="1803">
   <si>
     <t>type</t>
   </si>
@@ -5865,6 +5866,209 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7EB2CED5-68C7-4B05-97D5-B1E6F5C025C6}">
+  <dimension ref="A1:A38"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="43.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>580</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>589</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>597</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>609</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>619</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>637</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>661</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>677</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>678</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>685</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>741</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>750</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>774</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>818</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E00A43C7-5EDC-420A-BAE1-7DE9263A4D1A}">
   <dimension ref="A1:I304"/>
   <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
@@ -13466,7 +13670,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF8B3923-9D95-405B-A0EC-4AC4B020387B}">
   <dimension ref="A1:M195"/>
   <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
@@ -19683,7 +19887,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C6DC4AD-2D50-45A7-B323-E74BBFC6E484}">
   <dimension ref="A1:S219"/>
   <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
@@ -29270,7 +29474,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A623DF7-8824-47EF-81D7-78EB44C59BE6}">
   <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
@@ -29339,7 +29543,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2FC1A9E-6FD9-4DE2-9760-917D84C43308}">
   <dimension ref="A1:B29"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
@@ -29581,7 +29785,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6753FF9-DA34-424A-8D40-CFFBE1264805}">
   <dimension ref="A1:H334"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
@@ -36921,7 +37125,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0FD869C7-5BB3-42EF-8B5A-18BD78666649}">
   <dimension ref="A1:B1"/>
   <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>

</xml_diff>